<commit_message>
Absensi 17-18 Sept (TKa 5 mark: Evano17, Rachellyn/Hester/Hestine 17-18; TKB(2) Willian 17-18; TKB1 Kenzo 18)
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi T.P 2026-2027/Absensi 18 September 2026 Friday 09_45_34.xlsx
+++ b/PC-06/docs/Absensi T.P 2026-2027/Absensi 18 September 2026 Friday 09_45_34.xlsx
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW47"/>
+  <dimension ref="A1:AO47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -3754,7 +3754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AW51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -4560,7 +4560,11 @@
       </c>
       <c r="R16" s="8" t="n"/>
       <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
+      <c r="T16" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="U16" s="8" t="n"/>
       <c r="V16" s="8" t="n"/>
       <c r="W16" s="8" t="n"/>
@@ -4810,8 +4814,16 @@
           <t>S</t>
         </is>
       </c>
-      <c r="T21" s="8" t="n"/>
-      <c r="U21" s="8" t="n"/>
+      <c r="T21" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U21" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="V21" s="8" t="n"/>
       <c r="W21" s="8" t="n"/>
       <c r="X21" s="8" t="n"/>
@@ -4868,8 +4880,16 @@
           <t>S</t>
         </is>
       </c>
-      <c r="T22" s="8" t="n"/>
-      <c r="U22" s="8" t="n"/>
+      <c r="T22" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U22" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="V22" s="8" t="n"/>
       <c r="W22" s="8" t="n"/>
       <c r="X22" s="8" t="n"/>
@@ -5368,8 +5388,16 @@
           <t>S</t>
         </is>
       </c>
-      <c r="T32" s="8" t="n"/>
-      <c r="U32" s="8" t="n"/>
+      <c r="T32" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U32" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="V32" s="8" t="n"/>
       <c r="W32" s="8" t="n"/>
       <c r="X32" s="8" t="n"/>
@@ -8165,7 +8193,11 @@
       <c r="R21" s="8" t="n"/>
       <c r="S21" s="8" t="n"/>
       <c r="T21" s="8" t="n"/>
-      <c r="U21" s="8" t="n"/>
+      <c r="U21" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="V21" s="8" t="n"/>
       <c r="W21" s="8" t="n"/>
       <c r="X21" s="8" t="n"/>
@@ -11825,8 +11857,16 @@
           <t>S</t>
         </is>
       </c>
-      <c r="T29" s="8" t="n"/>
-      <c r="U29" s="8" t="n"/>
+      <c r="T29" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U29" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="V29" s="8" t="n"/>
       <c r="W29" s="8" t="n"/>
       <c r="X29" s="8" t="n"/>

</xml_diff>